<commit_message>
Output a completed Excel file with remove strivethrough cell.
Next: Filling the Boolean values for the three Auto Log columns.
</commit_message>
<xml_diff>
--- a/SWTest/Navigator.xlsx
+++ b/SWTest/Navigator.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\u245231\Quan_Vo\Local_Dev\complete-pandas-tutorial\SWTest\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96C55068-E879-44D4-A24C-8088C009132F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7E00F4F-E67E-4FB4-A1BB-B4F89A089B70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28800" yWindow="-7425" windowWidth="15870" windowHeight="11310" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Navigator" sheetId="1" r:id="rId1"/>
@@ -75,9 +75,6 @@
     <t>NA</t>
   </si>
   <si>
-    <t xml:space="preserve"> Log event if SOT (start of trip) slected</t>
-  </si>
-  <si>
     <t>0x04D2</t>
   </si>
   <si>
@@ -1011,6 +1008,9 @@
       <t xml:space="preserve">
 </t>
     </r>
+  </si>
+  <si>
+    <t>Log event if SOT (start of trip) slected</t>
   </si>
 </sst>
 </file>
@@ -1525,16 +1525,16 @@
   <sheetData>
     <row r="1" spans="1:10" s="1" customFormat="1" ht="25.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
+        <v>300</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>301</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>302</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>303</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>8</v>
@@ -1543,7 +1543,7 @@
         <v>1</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="H1" s="3" t="s">
         <v>2</v>
@@ -1581,16 +1581,16 @@
         <v>11</v>
       </c>
       <c r="I2" s="8" t="s">
-        <v>12</v>
+        <v>306</v>
       </c>
       <c r="J2" s="4"/>
     </row>
     <row r="3" spans="1:10" s="9" customFormat="1" ht="20.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="C3" s="4" t="s">
         <v>7</v>
@@ -1605,22 +1605,22 @@
         <v>9</v>
       </c>
       <c r="G3" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H3" s="7" t="s">
         <v>14</v>
-      </c>
-      <c r="H3" s="7" t="s">
-        <v>15</v>
       </c>
       <c r="I3" s="4"/>
       <c r="J3" s="8" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
     </row>
     <row r="4" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B4" s="4" t="s">
         <v>16</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>17</v>
       </c>
       <c r="C4" s="4" t="s">
         <v>7</v>
@@ -1641,19 +1641,19 @@
         <v>11</v>
       </c>
       <c r="I4" s="10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="J4"/>
     </row>
     <row r="5" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="B5" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="C5" s="4" t="s">
         <v>20</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>21</v>
       </c>
       <c r="D5" s="4" t="b">
         <v>1</v>
@@ -1674,41 +1674,41 @@
     </row>
     <row r="6" spans="1:10" s="9" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" s="11" t="s">
+        <v>21</v>
+      </c>
+      <c r="B6" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="C6" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D6" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="E6" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G6" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H6" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="C6" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="D6" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="E6" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="F6" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="G6" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="H6" s="12" t="s">
+      <c r="I6" s="8" t="s">
         <v>24</v>
-      </c>
-      <c r="I6" s="8" t="s">
-        <v>25</v>
       </c>
       <c r="J6" s="4"/>
     </row>
     <row r="7" spans="1:10" s="9" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="11" t="s">
+        <v>25</v>
+      </c>
+      <c r="B7" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="B7" s="6" t="s">
-        <v>27</v>
-      </c>
       <c r="C7" s="4" t="s">
         <v>7</v>
       </c>
@@ -1722,23 +1722,23 @@
         <v>9</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H7" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="I7" s="8" t="s">
         <v>24</v>
-      </c>
-      <c r="I7" s="8" t="s">
-        <v>25</v>
       </c>
       <c r="J7" s="4"/>
     </row>
     <row r="8" spans="1:10" s="9" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B8" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="B8" s="6" t="s">
-        <v>29</v>
-      </c>
       <c r="C8" s="4" t="s">
         <v>7</v>
       </c>
@@ -1752,83 +1752,83 @@
         <v>9</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H8" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="I8" s="8" t="s">
         <v>24</v>
-      </c>
-      <c r="I8" s="8" t="s">
-        <v>25</v>
       </c>
       <c r="J8" s="4"/>
     </row>
     <row r="9" spans="1:10" s="9" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="B9" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="C9" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D9" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="E9" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G9" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H9" s="12" t="s">
         <v>31</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="D9" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="E9" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="F9" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="G9" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="H9" s="12" t="s">
-        <v>32</v>
       </c>
       <c r="I9" s="4"/>
       <c r="J9" s="4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="10" spans="1:10" s="9" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="B10" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="C10" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D10" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="E10" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="F10" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G10" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H10" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="I10" s="8" t="s">
         <v>35</v>
-      </c>
-      <c r="C10" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="D10" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="E10" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="F10" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="G10" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="H10" s="12" t="s">
-        <v>32</v>
-      </c>
-      <c r="I10" s="8" t="s">
-        <v>36</v>
       </c>
       <c r="J10" s="4"/>
     </row>
     <row r="11" spans="1:10" s="9" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A11" s="11" t="s">
+        <v>36</v>
+      </c>
+      <c r="B11" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="B11" s="6" t="s">
-        <v>38</v>
-      </c>
       <c r="C11" s="4" t="s">
         <v>7</v>
       </c>
@@ -1842,23 +1842,23 @@
         <v>9</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H11" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="I11" s="8" t="s">
         <v>24</v>
-      </c>
-      <c r="I11" s="8" t="s">
-        <v>25</v>
       </c>
       <c r="J11" s="4"/>
     </row>
     <row r="12" spans="1:10" s="9" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A12" s="11" t="s">
+        <v>38</v>
+      </c>
+      <c r="B12" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="B12" s="6" t="s">
-        <v>40</v>
-      </c>
       <c r="C12" s="4" t="s">
         <v>7</v>
       </c>
@@ -1872,23 +1872,23 @@
         <v>9</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H12" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="I12" s="8" t="s">
         <v>24</v>
-      </c>
-      <c r="I12" s="8" t="s">
-        <v>25</v>
       </c>
       <c r="J12" s="4"/>
     </row>
     <row r="13" spans="1:10" s="9" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A13" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="B13" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="B13" s="6" t="s">
-        <v>42</v>
-      </c>
       <c r="C13" s="4" t="s">
         <v>7</v>
       </c>
@@ -1902,119 +1902,119 @@
         <v>9</v>
       </c>
       <c r="G13" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H13" s="12" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="I13" s="8" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="J13" s="4"/>
     </row>
     <row r="14" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="11" t="s">
+        <v>42</v>
+      </c>
+      <c r="B14" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="B14" s="4" t="s">
+      <c r="C14" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D14" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="E14" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="F14" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G14" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H14" s="7" t="s">
         <v>44</v>
-      </c>
-      <c r="C14" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="D14" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="E14" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="F14" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="G14" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="H14" s="7" t="s">
-        <v>45</v>
       </c>
       <c r="I14" s="4"/>
     </row>
     <row r="15" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="B15" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="B15" s="4" t="s">
+      <c r="C15" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D15" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="E15" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="F15" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G15" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="C15" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="D15" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="E15" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="F15" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="G15" s="4" t="s">
+      <c r="H15" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="I15" s="8" t="s">
         <v>48</v>
-      </c>
-      <c r="H15" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="I15" s="8" t="s">
-        <v>49</v>
       </c>
       <c r="J15" s="4"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="B16" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="B16" s="4" t="s">
+      <c r="C16" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D16" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="E16" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="F16" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G16" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H16" s="7" t="s">
         <v>51</v>
-      </c>
-      <c r="C16" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="D16" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="E16" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="F16" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="G16" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="H16" s="7" t="s">
-        <v>52</v>
       </c>
       <c r="I16" s="4"/>
       <c r="J16" s="9"/>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="B17" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="B17" s="4" t="s">
+      <c r="C17" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D17" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="E17" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="F17" s="4" t="s">
         <v>54</v>
-      </c>
-      <c r="C17" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="D17" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="E17" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="F17" s="4" t="s">
-        <v>55</v>
       </c>
       <c r="G17" s="4" t="s">
         <v>10</v>
@@ -2023,76 +2023,76 @@
         <v>108</v>
       </c>
       <c r="I17" s="8" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="J17" s="4"/>
     </row>
     <row r="18" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="B18" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="B18" s="4" t="s">
+      <c r="C18" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D18" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="E18" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="F18" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="C18" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="D18" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="E18" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="F18" s="4" t="s">
+      <c r="G18" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H18" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="G18" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="H18" s="7" t="s">
+      <c r="I18" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="I18" s="4" t="s">
+      <c r="J18" s="9" t="s">
         <v>61</v>
-      </c>
-      <c r="J18" s="9" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="19" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="11" t="s">
+        <v>62</v>
+      </c>
+      <c r="B19" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="B19" s="4" t="s">
+      <c r="C19" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D19" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="E19" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="F19" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G19" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H19" s="7" t="s">
         <v>64</v>
-      </c>
-      <c r="C19" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="D19" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="E19" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="F19" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="G19" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="H19" s="7" t="s">
-        <v>65</v>
       </c>
       <c r="I19" s="4"/>
     </row>
     <row r="20" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="B20" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="B20" s="4" t="s">
-        <v>67</v>
-      </c>
       <c r="C20" s="4" t="s">
         <v>7</v>
       </c>
@@ -2106,25 +2106,25 @@
         <v>9</v>
       </c>
       <c r="G20" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H20" s="7" t="s">
         <v>11</v>
       </c>
       <c r="I20" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="J20" s="4" t="s">
         <v>68</v>
-      </c>
-      <c r="J20" s="4" t="s">
-        <v>69</v>
       </c>
     </row>
     <row r="21" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="11" t="s">
+        <v>69</v>
+      </c>
+      <c r="B21" s="13" t="s">
         <v>70</v>
       </c>
-      <c r="B21" s="13" t="s">
-        <v>71</v>
-      </c>
       <c r="C21" s="4" t="s">
         <v>7</v>
       </c>
@@ -2138,7 +2138,7 @@
         <v>9</v>
       </c>
       <c r="G21" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="H21" s="7" t="s">
         <v>11</v>
@@ -2148,75 +2148,75 @@
     </row>
     <row r="22" spans="1:10" s="9" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A22" s="11" t="s">
+        <v>71</v>
+      </c>
+      <c r="B22" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="B22" s="4" t="s">
+      <c r="C22" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D22" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="E22" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="F22" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G22" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H22" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="I22" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="C22" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="D22" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="E22" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="F22" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="G22" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="H22" s="12" t="s">
-        <v>32</v>
-      </c>
-      <c r="I22" s="4" t="s">
+      <c r="J22" s="4" t="s">
         <v>74</v>
-      </c>
-      <c r="J22" s="4" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="23" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="11" t="s">
+        <v>75</v>
+      </c>
+      <c r="B23" t="s">
         <v>76</v>
       </c>
-      <c r="B23" t="s">
+      <c r="C23" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D23" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="E23" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="F23" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="C23" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="D23" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="E23" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="F23" s="4" t="s">
-        <v>78</v>
-      </c>
       <c r="G23" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="H23" s="7">
         <v>159</v>
       </c>
       <c r="I23" s="8" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="J23"/>
     </row>
     <row r="24" spans="1:10" s="9" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A24" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="B24" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="B24" s="4" t="s">
-        <v>81</v>
-      </c>
       <c r="C24" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D24" s="4" t="b">
         <v>1</v>
@@ -2228,54 +2228,54 @@
         <v>9</v>
       </c>
       <c r="G24" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H24" s="12" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="I24" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="J24" s="4" t="s">
         <v>74</v>
-      </c>
-      <c r="J24" s="4" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="25" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A25" s="11" t="s">
+        <v>81</v>
+      </c>
+      <c r="B25" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="B25" s="4" t="s">
+      <c r="C25" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D25" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="E25" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="F25" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G25" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H25" s="7" t="s">
         <v>83</v>
-      </c>
-      <c r="C25" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="D25" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="E25" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="F25" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="G25" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="H25" s="7" t="s">
-        <v>84</v>
       </c>
       <c r="I25" s="4"/>
     </row>
     <row r="26" spans="1:10" s="9" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A26" s="11" t="s">
+        <v>84</v>
+      </c>
+      <c r="B26" s="4" t="s">
         <v>85</v>
       </c>
-      <c r="B26" s="4" t="s">
-        <v>86</v>
-      </c>
       <c r="C26" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D26" s="4" t="b">
         <v>1</v>
@@ -2287,23 +2287,23 @@
         <v>9</v>
       </c>
       <c r="G26" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H26" s="12" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="I26" s="4"/>
       <c r="J26" s="4"/>
     </row>
     <row r="27" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A27" s="11" t="s">
+        <v>86</v>
+      </c>
+      <c r="B27" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="B27" s="4" t="s">
-        <v>88</v>
-      </c>
       <c r="C27" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D27" s="4" t="b">
         <v>1</v>
@@ -2315,53 +2315,53 @@
         <v>9</v>
       </c>
       <c r="G27" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H27" s="12" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="I27" s="4"/>
       <c r="J27" s="9"/>
     </row>
     <row r="28" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A28" s="11" t="s">
+        <v>88</v>
+      </c>
+      <c r="B28" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="B28" s="4" t="s">
+      <c r="C28" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D28" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="E28" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="F28" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G28" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H28" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="I28" s="8" t="s">
         <v>90</v>
-      </c>
-      <c r="C28" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="D28" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="E28" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="F28" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="G28" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="H28" s="12" t="s">
-        <v>32</v>
-      </c>
-      <c r="I28" s="8" t="s">
-        <v>91</v>
       </c>
       <c r="J28" s="4"/>
     </row>
     <row r="29" spans="1:10" s="9" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A29" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="B29" s="4" t="s">
         <v>92</v>
       </c>
-      <c r="B29" s="4" t="s">
-        <v>93</v>
-      </c>
       <c r="C29" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D29" s="4" t="b">
         <v>1</v>
@@ -2373,25 +2373,25 @@
         <v>9</v>
       </c>
       <c r="G29" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H29" s="12" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="I29" s="4"/>
       <c r="J29" s="4" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="30" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A30" s="11" t="s">
+        <v>94</v>
+      </c>
+      <c r="B30" s="4" t="s">
         <v>95</v>
       </c>
-      <c r="B30" s="4" t="s">
-        <v>96</v>
-      </c>
       <c r="C30" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D30" s="4" t="b">
         <v>1</v>
@@ -2412,13 +2412,13 @@
     </row>
     <row r="31" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A31" s="11" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D31" s="4" t="b">
         <v>1</v>
@@ -2430,23 +2430,23 @@
         <v>9</v>
       </c>
       <c r="G31" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H31" s="7" t="s">
         <v>11</v>
       </c>
       <c r="I31" s="4"/>
       <c r="J31" s="9" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
     </row>
     <row r="32" spans="1:10" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="11" t="s">
+        <v>97</v>
+      </c>
+      <c r="B32" s="13" t="s">
         <v>98</v>
       </c>
-      <c r="B32" s="13" t="s">
-        <v>99</v>
-      </c>
       <c r="C32" s="4" t="s">
         <v>7</v>
       </c>
@@ -2460,22 +2460,22 @@
         <v>9</v>
       </c>
       <c r="G32" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H32" s="12" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="I32" s="8" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="33" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A33" s="11" t="s">
+        <v>99</v>
+      </c>
+      <c r="B33" s="13" t="s">
         <v>100</v>
       </c>
-      <c r="B33" s="13" t="s">
-        <v>101</v>
-      </c>
       <c r="C33" s="4" t="s">
         <v>7</v>
       </c>
@@ -2489,52 +2489,52 @@
         <v>9</v>
       </c>
       <c r="G33" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H33" s="7" t="s">
         <v>11</v>
       </c>
       <c r="I33" s="8" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="J33"/>
     </row>
     <row r="34" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A34" s="11" t="s">
+        <v>102</v>
+      </c>
+      <c r="B34" s="6" t="s">
         <v>103</v>
       </c>
-      <c r="B34" s="6" t="s">
+      <c r="C34" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D34" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="E34" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="F34" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G34" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H34" s="12" t="s">
         <v>104</v>
       </c>
-      <c r="C34" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="D34" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="E34" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="F34" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="G34" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="H34" s="12" t="s">
+      <c r="I34" s="8" t="s">
         <v>105</v>
-      </c>
-      <c r="I34" s="8" t="s">
-        <v>106</v>
       </c>
       <c r="J34" s="4"/>
     </row>
     <row r="35" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A35" s="11" t="s">
+        <v>106</v>
+      </c>
+      <c r="B35" s="6" t="s">
         <v>107</v>
-      </c>
-      <c r="B35" s="6" t="s">
-        <v>108</v>
       </c>
       <c r="C35" s="4" t="s">
         <v>7</v>
@@ -2555,18 +2555,18 @@
         <v>11</v>
       </c>
       <c r="I35" s="8" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="J35" s="4" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="36" spans="1:10" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A36" s="11" t="s">
+        <v>109</v>
+      </c>
+      <c r="B36" s="6" t="s">
         <v>110</v>
-      </c>
-      <c r="B36" s="6" t="s">
-        <v>111</v>
       </c>
       <c r="C36" s="4" t="s">
         <v>7</v>
@@ -2587,18 +2587,18 @@
         <v>11</v>
       </c>
       <c r="I36" s="8" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="J36" s="4" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="37" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A37" s="11" t="s">
+        <v>111</v>
+      </c>
+      <c r="B37" s="6" t="s">
         <v>112</v>
-      </c>
-      <c r="B37" s="6" t="s">
-        <v>113</v>
       </c>
       <c r="C37" s="4" t="s">
         <v>7</v>
@@ -2619,18 +2619,18 @@
         <v>11</v>
       </c>
       <c r="I37" s="8" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="J37" s="4" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="38" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A38" s="11" t="s">
+        <v>113</v>
+      </c>
+      <c r="B38" s="4" t="s">
         <v>114</v>
-      </c>
-      <c r="B38" s="4" t="s">
-        <v>115</v>
       </c>
       <c r="C38" s="4" t="s">
         <v>7</v>
@@ -2651,16 +2651,16 @@
         <v>108</v>
       </c>
       <c r="I38" s="8" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="J38"/>
     </row>
     <row r="39" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A39" s="11" t="s">
+        <v>116</v>
+      </c>
+      <c r="B39" s="6" t="s">
         <v>117</v>
-      </c>
-      <c r="B39" s="6" t="s">
-        <v>118</v>
       </c>
       <c r="C39" s="4" t="s">
         <v>7</v>
@@ -2681,18 +2681,18 @@
         <v>11</v>
       </c>
       <c r="I39" s="8" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="J39" s="4" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="40" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A40" s="11" t="s">
+        <v>275</v>
+      </c>
+      <c r="B40" s="6" t="s">
         <v>276</v>
-      </c>
-      <c r="B40" s="6" t="s">
-        <v>277</v>
       </c>
       <c r="C40" s="4" t="s">
         <v>7</v>
@@ -2713,18 +2713,18 @@
         <v>11</v>
       </c>
       <c r="I40" s="8" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="J40" s="4" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="41" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A41" s="11" t="s">
+        <v>118</v>
+      </c>
+      <c r="B41" s="13" t="s">
         <v>119</v>
-      </c>
-      <c r="B41" s="13" t="s">
-        <v>120</v>
       </c>
       <c r="C41" s="4" t="s">
         <v>7</v>
@@ -2745,46 +2745,46 @@
         <v>66</v>
       </c>
       <c r="I41" s="4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="J41"/>
     </row>
     <row r="42" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A42" s="11" t="s">
+        <v>120</v>
+      </c>
+      <c r="B42" s="4" t="s">
         <v>121</v>
       </c>
-      <c r="B42" s="4" t="s">
+      <c r="C42" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D42" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="E42" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="F42" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G42" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="H42" s="7" t="s">
         <v>122</v>
       </c>
-      <c r="C42" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="D42" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="E42" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="F42" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="G42" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="H42" s="7" t="s">
+      <c r="I42" s="8" t="s">
         <v>123</v>
-      </c>
-      <c r="I42" s="8" t="s">
-        <v>124</v>
       </c>
       <c r="J42" s="4"/>
     </row>
     <row r="43" spans="1:10" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A43" s="11" t="s">
+        <v>124</v>
+      </c>
+      <c r="B43" s="6" t="s">
         <v>125</v>
-      </c>
-      <c r="B43" s="6" t="s">
-        <v>126</v>
       </c>
       <c r="C43" s="4" t="s">
         <v>7</v>
@@ -2805,18 +2805,18 @@
         <v>11</v>
       </c>
       <c r="I43" s="8" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="J43" s="4" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="44" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A44" s="11" t="s">
+        <v>126</v>
+      </c>
+      <c r="B44" s="13" t="s">
         <v>127</v>
-      </c>
-      <c r="B44" s="13" t="s">
-        <v>128</v>
       </c>
       <c r="C44" s="4" t="s">
         <v>7</v>
@@ -2834,18 +2834,18 @@
         <v>10</v>
       </c>
       <c r="H44" s="7" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="I44" s="4"/>
       <c r="J44"/>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A45" s="11" t="s">
+        <v>129</v>
+      </c>
+      <c r="B45" s="13" t="s">
         <v>130</v>
       </c>
-      <c r="B45" s="13" t="s">
-        <v>131</v>
-      </c>
       <c r="C45" s="4" t="s">
         <v>7</v>
       </c>
@@ -2859,24 +2859,24 @@
         <v>9</v>
       </c>
       <c r="G45" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H45" s="7" t="s">
         <v>11</v>
       </c>
       <c r="I45" s="8" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A46" s="11" t="s">
+        <v>132</v>
+      </c>
+      <c r="B46" s="4" t="s">
         <v>133</v>
       </c>
-      <c r="B46" s="4" t="s">
-        <v>134</v>
-      </c>
       <c r="C46" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D46" s="4" t="b">
         <v>1</v>
@@ -2891,105 +2891,105 @@
         <v>10</v>
       </c>
       <c r="H46" s="7" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="I46" s="4"/>
       <c r="J46" s="9"/>
     </row>
     <row r="47" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A47" s="11" t="s">
+        <v>135</v>
+      </c>
+      <c r="B47" s="4" t="s">
         <v>136</v>
       </c>
-      <c r="B47" s="4" t="s">
+      <c r="C47" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D47" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="E47" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="F47" s="4" t="s">
         <v>137</v>
       </c>
-      <c r="C47" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="D47" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="E47" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="F47" s="4" t="s">
+      <c r="G47" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H47" s="7" t="s">
         <v>138</v>
-      </c>
-      <c r="G47" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="H47" s="7" t="s">
-        <v>139</v>
       </c>
       <c r="I47" s="4"/>
       <c r="J47" s="9"/>
     </row>
     <row r="48" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A48" s="11" t="s">
+        <v>139</v>
+      </c>
+      <c r="B48" s="13" t="s">
         <v>140</v>
       </c>
-      <c r="B48" s="13" t="s">
+      <c r="C48" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D48" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="E48" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="F48" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="G48" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H48" s="7">
+        <v>7</v>
+      </c>
+      <c r="I48" s="4" t="s">
         <v>141</v>
-      </c>
-      <c r="C48" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="D48" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="E48" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="F48" s="4" t="s">
-        <v>138</v>
-      </c>
-      <c r="G48" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="H48" s="7">
-        <v>7</v>
-      </c>
-      <c r="I48" s="4" t="s">
-        <v>142</v>
       </c>
     </row>
     <row r="49" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A49" s="11" t="s">
+        <v>142</v>
+      </c>
+      <c r="B49" s="4" t="s">
         <v>143</v>
       </c>
-      <c r="B49" s="4" t="s">
+      <c r="C49" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D49" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="E49" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="F49" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="G49" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H49" s="7" t="s">
         <v>144</v>
-      </c>
-      <c r="C49" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="D49" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="E49" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="F49" s="4" t="s">
-        <v>138</v>
-      </c>
-      <c r="G49" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="H49" s="7" t="s">
-        <v>145</v>
       </c>
       <c r="I49" s="4"/>
       <c r="J49" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="50" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A50" s="11" t="s">
+        <v>146</v>
+      </c>
+      <c r="B50" s="4" t="s">
         <v>147</v>
       </c>
-      <c r="B50" s="4" t="s">
-        <v>148</v>
-      </c>
       <c r="C50" s="4" t="s">
         <v>7</v>
       </c>
@@ -3000,26 +3000,26 @@
         <v>1</v>
       </c>
       <c r="F50" s="4" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="G50" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="H50" s="7" t="s">
+        <v>122</v>
+      </c>
+      <c r="I50" s="8" t="s">
         <v>48</v>
-      </c>
-      <c r="H50" s="7" t="s">
-        <v>123</v>
-      </c>
-      <c r="I50" s="8" t="s">
-        <v>49</v>
       </c>
       <c r="J50" s="4"/>
     </row>
     <row r="51" spans="1:10" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A51" s="11" t="s">
+        <v>148</v>
+      </c>
+      <c r="B51" s="4" t="s">
         <v>149</v>
       </c>
-      <c r="B51" s="4" t="s">
-        <v>150</v>
-      </c>
       <c r="C51" s="4" t="s">
         <v>7</v>
       </c>
@@ -3030,10 +3030,10 @@
         <v>0</v>
       </c>
       <c r="F51" s="4" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="G51" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H51" s="15"/>
       <c r="I51" s="4"/>
@@ -3041,11 +3041,11 @@
     </row>
     <row r="52" spans="1:10" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A52" s="11" t="s">
+        <v>150</v>
+      </c>
+      <c r="B52" s="13" t="s">
         <v>151</v>
       </c>
-      <c r="B52" s="13" t="s">
-        <v>152</v>
-      </c>
       <c r="C52" s="4" t="s">
         <v>7</v>
       </c>
@@ -3056,26 +3056,26 @@
         <v>1</v>
       </c>
       <c r="F52" s="4" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="G52" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H52" s="7">
         <v>15</v>
       </c>
       <c r="I52" s="8" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="J52"/>
     </row>
     <row r="53" spans="1:10" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A53" s="11" t="s">
+        <v>152</v>
+      </c>
+      <c r="B53" s="13" t="s">
         <v>153</v>
       </c>
-      <c r="B53" s="13" t="s">
-        <v>154</v>
-      </c>
       <c r="C53" s="4" t="s">
         <v>7</v>
       </c>
@@ -3086,85 +3086,85 @@
         <v>1</v>
       </c>
       <c r="F53" s="4" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="G53" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H53" s="7">
         <v>629</v>
       </c>
       <c r="I53" s="4" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="J53" s="4"/>
     </row>
     <row r="54" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A54" s="11" t="s">
+        <v>155</v>
+      </c>
+      <c r="B54" s="4" t="s">
         <v>156</v>
       </c>
-      <c r="B54" s="4" t="s">
+      <c r="C54" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D54" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="E54" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="F54" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G54" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H54" s="7" t="s">
         <v>157</v>
       </c>
-      <c r="C54" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="D54" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="E54" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="F54" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="G54" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="H54" s="7" t="s">
+      <c r="I54" s="8" t="s">
         <v>158</v>
-      </c>
-      <c r="I54" s="8" t="s">
-        <v>159</v>
       </c>
     </row>
     <row r="55" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A55" s="11" t="s">
+        <v>159</v>
+      </c>
+      <c r="B55" s="4" t="s">
         <v>160</v>
       </c>
-      <c r="B55" s="4" t="s">
+      <c r="C55" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D55" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="E55" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="F55" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G55" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="H55" s="7" t="s">
         <v>161</v>
       </c>
-      <c r="C55" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="D55" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="E55" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="F55" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="G55" s="4" t="s">
+      <c r="I55" s="8" t="s">
         <v>48</v>
-      </c>
-      <c r="H55" s="7" t="s">
-        <v>162</v>
-      </c>
-      <c r="I55" s="8" t="s">
-        <v>49</v>
       </c>
       <c r="J55" s="4"/>
     </row>
     <row r="56" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A56" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="B56" s="4" t="s">
         <v>163</v>
       </c>
-      <c r="B56" s="4" t="s">
-        <v>164</v>
-      </c>
       <c r="C56" s="4" t="s">
         <v>7</v>
       </c>
@@ -3178,54 +3178,54 @@
         <v>9</v>
       </c>
       <c r="G56" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H56" s="7" t="s">
         <v>11</v>
       </c>
       <c r="I56" s="10" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="57" spans="1:10" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="11" t="s">
+        <v>165</v>
+      </c>
+      <c r="B57" s="4" t="s">
         <v>166</v>
       </c>
-      <c r="B57" s="4" t="s">
+      <c r="C57" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D57" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="E57" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="F57" s="8" t="s">
+        <v>293</v>
+      </c>
+      <c r="G57" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H57" s="7" t="s">
         <v>167</v>
       </c>
-      <c r="C57" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="D57" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="E57" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="F57" s="8" t="s">
-        <v>294</v>
-      </c>
-      <c r="G57" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="H57" s="7" t="s">
-        <v>168</v>
-      </c>
       <c r="I57" s="8" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="J57" s="8" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
     </row>
     <row r="58" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A58" s="11" t="s">
+        <v>169</v>
+      </c>
+      <c r="B58" s="4" t="s">
         <v>170</v>
       </c>
-      <c r="B58" s="4" t="s">
-        <v>171</v>
-      </c>
       <c r="C58" s="4" t="s">
         <v>7</v>
       </c>
@@ -3239,85 +3239,85 @@
         <v>9</v>
       </c>
       <c r="G58" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="H58" s="7" t="s">
+        <v>122</v>
+      </c>
+      <c r="I58" s="8" t="s">
         <v>48</v>
-      </c>
-      <c r="H58" s="7" t="s">
-        <v>123</v>
-      </c>
-      <c r="I58" s="8" t="s">
-        <v>49</v>
       </c>
       <c r="J58" s="4"/>
     </row>
     <row r="59" spans="1:10" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59" s="11" t="s">
+        <v>171</v>
+      </c>
+      <c r="B59" s="4" t="s">
         <v>172</v>
       </c>
-      <c r="B59" s="4" t="s">
+      <c r="C59" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D59" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="E59" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="F59" s="8" t="s">
+        <v>293</v>
+      </c>
+      <c r="G59" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H59" s="7" t="s">
         <v>173</v>
       </c>
-      <c r="C59" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="D59" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="E59" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="F59" s="8" t="s">
+      <c r="I59" s="8" t="s">
+        <v>174</v>
+      </c>
+      <c r="J59" s="9" t="s">
         <v>294</v>
-      </c>
-      <c r="G59" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="H59" s="7" t="s">
-        <v>174</v>
-      </c>
-      <c r="I59" s="8" t="s">
-        <v>175</v>
-      </c>
-      <c r="J59" s="9" t="s">
-        <v>295</v>
       </c>
     </row>
     <row r="60" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A60" s="11" t="s">
+        <v>175</v>
+      </c>
+      <c r="B60" s="4" t="s">
         <v>176</v>
       </c>
-      <c r="B60" s="4" t="s">
+      <c r="C60" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D60" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="E60" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="F60" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G60" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H60" s="7" t="s">
         <v>177</v>
       </c>
-      <c r="C60" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="D60" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="E60" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="F60" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="G60" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="H60" s="7" t="s">
-        <v>178</v>
-      </c>
       <c r="I60" s="8" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="J60" s="9"/>
     </row>
     <row r="61" spans="1:10" ht="75" x14ac:dyDescent="0.25">
       <c r="A61" s="11" t="s">
+        <v>178</v>
+      </c>
+      <c r="B61" s="4" t="s">
         <v>179</v>
       </c>
-      <c r="B61" s="4" t="s">
-        <v>180</v>
-      </c>
       <c r="C61" s="4" t="s">
         <v>7</v>
       </c>
@@ -3328,60 +3328,60 @@
         <v>1</v>
       </c>
       <c r="F61" s="8" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="G61" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H61" s="7" t="s">
         <v>11</v>
       </c>
       <c r="I61" s="8" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="J61" s="19" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
     </row>
     <row r="62" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A62" s="11" t="s">
+        <v>181</v>
+      </c>
+      <c r="B62" s="4" t="s">
         <v>182</v>
       </c>
-      <c r="B62" s="4" t="s">
+      <c r="C62" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D62" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="E62" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="F62" s="4" t="s">
         <v>183</v>
       </c>
-      <c r="C62" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="D62" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="E62" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="F62" s="4" t="s">
-        <v>184</v>
-      </c>
       <c r="G62" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H62" s="7">
         <v>40</v>
       </c>
       <c r="I62" s="8" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="J62" s="9"/>
     </row>
     <row r="63" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A63" s="11" t="s">
+        <v>185</v>
+      </c>
+      <c r="B63" s="4" t="s">
         <v>186</v>
       </c>
-      <c r="B63" s="4" t="s">
-        <v>187</v>
-      </c>
       <c r="C63" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D63" s="4" t="b">
         <v>1</v>
@@ -3393,53 +3393,53 @@
         <v>9</v>
       </c>
       <c r="G63" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H63" s="12" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="I63" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="J63" s="4" t="s">
         <v>74</v>
-      </c>
-      <c r="J63" s="4" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="64" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A64" s="11" t="s">
+        <v>187</v>
+      </c>
+      <c r="B64" s="4" t="s">
         <v>188</v>
       </c>
-      <c r="B64" s="4" t="s">
+      <c r="C64" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D64" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="E64" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="F64" s="4" t="s">
+        <v>183</v>
+      </c>
+      <c r="G64" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H64" s="7" t="s">
         <v>189</v>
-      </c>
-      <c r="C64" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="D64" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="E64" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="F64" s="4" t="s">
-        <v>184</v>
-      </c>
-      <c r="G64" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="H64" s="7" t="s">
-        <v>190</v>
       </c>
       <c r="I64" s="4"/>
       <c r="J64" s="9"/>
     </row>
     <row r="65" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A65" s="11" t="s">
+        <v>190</v>
+      </c>
+      <c r="B65" s="4" t="s">
         <v>191</v>
       </c>
-      <c r="B65" s="4" t="s">
-        <v>192</v>
-      </c>
       <c r="C65" s="4" t="s">
         <v>7</v>
       </c>
@@ -3453,24 +3453,24 @@
         <v>9</v>
       </c>
       <c r="G65" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H65" s="7">
         <v>111</v>
       </c>
       <c r="I65" s="8" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="66" spans="1:10" s="9" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A66" s="11" t="s">
+        <v>193</v>
+      </c>
+      <c r="B66" s="4" t="s">
         <v>194</v>
       </c>
-      <c r="B66" s="4" t="s">
-        <v>195</v>
-      </c>
       <c r="C66" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D66" s="4" t="b">
         <v>1</v>
@@ -3482,54 +3482,54 @@
         <v>9</v>
       </c>
       <c r="G66" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H66" s="12" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="I66" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="J66" s="4" t="s">
         <v>74</v>
-      </c>
-      <c r="J66" s="4" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="67" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A67" s="11" t="s">
+        <v>195</v>
+      </c>
+      <c r="B67" s="4" t="s">
         <v>196</v>
       </c>
-      <c r="B67" s="4" t="s">
+      <c r="C67" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D67" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="E67" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="F67" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G67" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H67" s="7" t="s">
         <v>197</v>
       </c>
-      <c r="C67" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="D67" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="E67" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="F67" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="G67" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="H67" s="7" t="s">
+      <c r="I67" s="8" t="s">
         <v>198</v>
-      </c>
-      <c r="I67" s="8" t="s">
-        <v>199</v>
       </c>
     </row>
     <row r="68" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A68" s="11" t="s">
+        <v>199</v>
+      </c>
+      <c r="B68" s="4" t="s">
         <v>200</v>
       </c>
-      <c r="B68" s="4" t="s">
-        <v>201</v>
-      </c>
       <c r="C68" s="4" t="s">
         <v>7</v>
       </c>
@@ -3543,21 +3543,21 @@
         <v>9</v>
       </c>
       <c r="G68" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H68" s="7" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="I68" s="4"/>
       <c r="J68" s="9"/>
     </row>
     <row r="69" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A69" s="11" t="s">
+        <v>201</v>
+      </c>
+      <c r="B69" s="4" t="s">
         <v>202</v>
       </c>
-      <c r="B69" s="4" t="s">
-        <v>203</v>
-      </c>
       <c r="C69" s="4" t="s">
         <v>7</v>
       </c>
@@ -3571,22 +3571,22 @@
         <v>9</v>
       </c>
       <c r="G69" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="H69" s="7">
         <v>89</v>
       </c>
       <c r="I69" s="4" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="J69" s="9"/>
     </row>
     <row r="70" spans="1:10" ht="69" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A70" s="20" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="B70" s="21" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="C70" s="22" t="s">
         <v>7</v>
@@ -3607,19 +3607,19 @@
         <v>66</v>
       </c>
       <c r="I70" s="24" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="J70" s="9" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
     </row>
     <row r="71" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A71" s="11" t="s">
+        <v>205</v>
+      </c>
+      <c r="B71" s="13" t="s">
         <v>206</v>
       </c>
-      <c r="B71" s="13" t="s">
-        <v>207</v>
-      </c>
       <c r="C71" s="4" t="s">
         <v>7</v>
       </c>
@@ -3633,24 +3633,24 @@
         <v>9</v>
       </c>
       <c r="G71" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H71" s="7" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="I71" s="8" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="72" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A72" s="11" t="s">
+        <v>207</v>
+      </c>
+      <c r="B72" s="4" t="s">
         <v>208</v>
       </c>
-      <c r="B72" s="4" t="s">
-        <v>209</v>
-      </c>
       <c r="C72" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D72" s="4" t="b">
         <v>1</v>
@@ -3659,26 +3659,26 @@
         <v>0</v>
       </c>
       <c r="F72" s="4" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="G72" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H72" s="7" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="I72" s="4"/>
       <c r="J72" s="4" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="73" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A73" s="5" t="s">
+        <v>210</v>
+      </c>
+      <c r="B73" s="4" t="s">
         <v>211</v>
       </c>
-      <c r="B73" s="4" t="s">
-        <v>212</v>
-      </c>
       <c r="C73" s="4" t="s">
         <v>7</v>
       </c>
@@ -3689,87 +3689,87 @@
         <v>1</v>
       </c>
       <c r="F73" s="8" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="G73" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H73" s="7" t="s">
         <v>11</v>
       </c>
       <c r="I73" s="10" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="J73" s="9" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
     </row>
     <row r="74" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A74" s="11" t="s">
+        <v>212</v>
+      </c>
+      <c r="B74" s="4" t="s">
         <v>213</v>
       </c>
-      <c r="B74" s="4" t="s">
+      <c r="C74" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D74" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="E74" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="F74" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G74" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H74" s="12" t="s">
         <v>214</v>
-      </c>
-      <c r="C74" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="D74" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="E74" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="F74" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="G74" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="H74" s="12" t="s">
-        <v>215</v>
       </c>
       <c r="I74" s="4"/>
       <c r="J74" s="9"/>
     </row>
     <row r="75" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A75" s="11" t="s">
+        <v>215</v>
+      </c>
+      <c r="B75" s="4" t="s">
         <v>216</v>
       </c>
-      <c r="B75" s="4" t="s">
+      <c r="C75" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D75" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="E75" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="F75" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G75" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H75" s="7" t="s">
         <v>217</v>
       </c>
-      <c r="C75" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="D75" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="E75" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="F75" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="G75" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="H75" s="7" t="s">
-        <v>218</v>
-      </c>
       <c r="I75" s="8" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="J75" s="4" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="76" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A76" s="11" t="s">
+        <v>218</v>
+      </c>
+      <c r="B76" s="4" t="s">
         <v>219</v>
-      </c>
-      <c r="B76" s="4" t="s">
-        <v>220</v>
       </c>
       <c r="C76" s="4" t="s">
         <v>7</v>
@@ -3787,17 +3787,17 @@
         <v>10</v>
       </c>
       <c r="H76" s="7" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="I76" s="4"/>
       <c r="J76" s="9"/>
     </row>
     <row r="77" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A77" s="5" t="s">
+        <v>220</v>
+      </c>
+      <c r="B77" s="6" t="s">
         <v>221</v>
-      </c>
-      <c r="B77" s="6" t="s">
-        <v>222</v>
       </c>
       <c r="C77" s="4" t="s">
         <v>7</v>
@@ -3818,16 +3818,16 @@
         <v>11</v>
       </c>
       <c r="I77" s="8" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="J77" s="4"/>
     </row>
     <row r="78" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A78" s="11" t="s">
+        <v>223</v>
+      </c>
+      <c r="B78" s="6" t="s">
         <v>224</v>
-      </c>
-      <c r="B78" s="6" t="s">
-        <v>225</v>
       </c>
       <c r="C78" s="4" t="s">
         <v>7</v>
@@ -3848,19 +3848,19 @@
         <v>11</v>
       </c>
       <c r="I78" s="8" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="J78" s="4"/>
     </row>
     <row r="79" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A79" s="11" t="s">
+        <v>226</v>
+      </c>
+      <c r="B79" s="4" t="s">
         <v>227</v>
       </c>
-      <c r="B79" s="4" t="s">
-        <v>228</v>
-      </c>
       <c r="C79" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D79" s="4" t="b">
         <v>1</v>
@@ -3882,13 +3882,13 @@
     </row>
     <row r="80" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A80" s="11" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="B80" s="4" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="C80" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D80" s="4" t="b">
         <v>1</v>
@@ -3900,23 +3900,23 @@
         <v>9</v>
       </c>
       <c r="G80" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H80" s="7" t="s">
         <v>11</v>
       </c>
       <c r="I80" s="4"/>
       <c r="J80" s="9" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
     </row>
     <row r="81" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A81" s="11" t="s">
+        <v>229</v>
+      </c>
+      <c r="B81" t="s">
         <v>230</v>
       </c>
-      <c r="B81" t="s">
-        <v>231</v>
-      </c>
       <c r="C81" s="4" t="s">
         <v>7</v>
       </c>
@@ -3927,25 +3927,25 @@
         <v>1</v>
       </c>
       <c r="F81" s="4" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="G81" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="H81" s="7">
         <v>159</v>
       </c>
       <c r="I81" s="8" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="82" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A82" s="11" t="s">
+        <v>231</v>
+      </c>
+      <c r="B82" s="4" t="s">
         <v>232</v>
       </c>
-      <c r="B82" s="4" t="s">
-        <v>233</v>
-      </c>
       <c r="C82" s="4" t="s">
         <v>7</v>
       </c>
@@ -3959,23 +3959,23 @@
         <v>9</v>
       </c>
       <c r="G82" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="H82" s="7" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="I82" s="4" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="J82" s="4"/>
     </row>
     <row r="83" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A83" s="11" t="s">
+        <v>233</v>
+      </c>
+      <c r="B83" s="4" t="s">
         <v>234</v>
       </c>
-      <c r="B83" s="4" t="s">
-        <v>235</v>
-      </c>
       <c r="C83" s="4" t="s">
         <v>7</v>
       </c>
@@ -3989,23 +3989,23 @@
         <v>9</v>
       </c>
       <c r="G83" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H83" s="7">
         <v>159</v>
       </c>
       <c r="I83" s="8" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="J83" s="4"/>
     </row>
     <row r="84" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A84" s="11" t="s">
+        <v>236</v>
+      </c>
+      <c r="B84" s="4" t="s">
         <v>237</v>
       </c>
-      <c r="B84" s="4" t="s">
-        <v>238</v>
-      </c>
       <c r="C84" s="4" t="s">
         <v>7</v>
       </c>
@@ -4019,23 +4019,23 @@
         <v>9</v>
       </c>
       <c r="G84" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H84" s="7">
         <v>159</v>
       </c>
       <c r="I84" s="8" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="J84" s="4"/>
     </row>
     <row r="85" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A85" s="11" t="s">
+        <v>238</v>
+      </c>
+      <c r="B85" s="4" t="s">
         <v>239</v>
       </c>
-      <c r="B85" s="4" t="s">
-        <v>240</v>
-      </c>
       <c r="C85" s="4" t="s">
         <v>7</v>
       </c>
@@ -4049,23 +4049,23 @@
         <v>9</v>
       </c>
       <c r="G85" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H85" s="7">
         <v>159</v>
       </c>
       <c r="I85" s="8" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="J85" s="4"/>
     </row>
     <row r="86" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A86" s="11" t="s">
+        <v>241</v>
+      </c>
+      <c r="B86" s="4" t="s">
         <v>242</v>
       </c>
-      <c r="B86" s="4" t="s">
-        <v>243</v>
-      </c>
       <c r="C86" s="4" t="s">
         <v>7</v>
       </c>
@@ -4079,24 +4079,24 @@
         <v>9</v>
       </c>
       <c r="G86" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H86" s="7">
         <v>159</v>
       </c>
       <c r="I86" s="8" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
     </row>
     <row r="87" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A87" s="11" t="s">
+        <v>243</v>
+      </c>
+      <c r="B87" s="4" t="s">
         <v>244</v>
       </c>
-      <c r="B87" s="4" t="s">
-        <v>245</v>
-      </c>
       <c r="C87" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D87" s="4" t="b">
         <v>1</v>
@@ -4108,24 +4108,24 @@
         <v>9</v>
       </c>
       <c r="G87" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H87" s="7" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="I87" s="4"/>
       <c r="J87" s="4"/>
     </row>
     <row r="88" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A88" s="11" t="s">
+        <v>245</v>
+      </c>
+      <c r="B88" s="13" t="s">
         <v>246</v>
       </c>
-      <c r="B88" s="13" t="s">
+      <c r="C88" s="4" t="s">
         <v>247</v>
       </c>
-      <c r="C88" s="4" t="s">
-        <v>248</v>
-      </c>
       <c r="D88" s="4" t="b">
         <v>1</v>
       </c>
@@ -4136,7 +4136,7 @@
         <v>9</v>
       </c>
       <c r="G88" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H88" s="7">
         <v>33</v>
@@ -4145,22 +4145,22 @@
     </row>
     <row r="89" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A89" s="11" t="s">
+        <v>248</v>
+      </c>
+      <c r="B89" s="4" t="s">
         <v>249</v>
       </c>
-      <c r="B89" s="4" t="s">
+      <c r="C89" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D89" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="E89" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="F89" s="4" t="s">
         <v>250</v>
-      </c>
-      <c r="C89" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="D89" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="E89" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="F89" s="4" t="s">
-        <v>251</v>
       </c>
       <c r="G89" s="4" t="s">
         <v>10</v>
@@ -4169,21 +4169,21 @@
         <v>49</v>
       </c>
       <c r="I89" s="4" t="s">
+        <v>251</v>
+      </c>
+      <c r="J89" s="4" t="s">
         <v>252</v>
-      </c>
-      <c r="J89" s="4" t="s">
-        <v>253</v>
       </c>
     </row>
     <row r="90" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A90" s="11" t="s">
+        <v>253</v>
+      </c>
+      <c r="B90" s="4" t="s">
         <v>254</v>
       </c>
-      <c r="B90" s="4" t="s">
-        <v>255</v>
-      </c>
       <c r="C90" s="4" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="D90" s="4" t="b">
         <v>1</v>
@@ -4205,11 +4205,11 @@
     </row>
     <row r="91" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A91" s="11" t="s">
+        <v>255</v>
+      </c>
+      <c r="B91" s="13" t="s">
         <v>256</v>
       </c>
-      <c r="B91" s="13" t="s">
-        <v>257</v>
-      </c>
       <c r="C91" s="4" t="s">
         <v>7</v>
       </c>
@@ -4223,20 +4223,20 @@
         <v>9</v>
       </c>
       <c r="G91" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H91" s="7" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="I91" s="4"/>
     </row>
     <row r="92" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A92" s="11" t="s">
+        <v>257</v>
+      </c>
+      <c r="B92" s="4" t="s">
         <v>258</v>
       </c>
-      <c r="B92" s="4" t="s">
-        <v>259</v>
-      </c>
       <c r="C92" s="4" t="s">
         <v>7</v>
       </c>
@@ -4250,54 +4250,54 @@
         <v>9</v>
       </c>
       <c r="G92" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H92" s="7">
         <v>111</v>
       </c>
       <c r="I92" s="8" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
     </row>
     <row r="93" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A93" s="11" t="s">
+        <v>260</v>
+      </c>
+      <c r="B93" s="4" t="s">
         <v>261</v>
       </c>
-      <c r="B93" s="4" t="s">
+      <c r="C93" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D93" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="E93" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="F93" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G93" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H93" s="7" t="s">
         <v>262</v>
       </c>
-      <c r="C93" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="D93" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="E93" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="F93" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="G93" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="H93" s="7" t="s">
-        <v>263</v>
-      </c>
       <c r="I93" s="8" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="J93" s="4" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="94" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A94" s="11" t="s">
+        <v>263</v>
+      </c>
+      <c r="B94" s="4" t="s">
         <v>264</v>
       </c>
-      <c r="B94" s="4" t="s">
-        <v>265</v>
-      </c>
       <c r="C94" s="4" t="s">
         <v>7</v>
       </c>
@@ -4311,53 +4311,53 @@
         <v>9</v>
       </c>
       <c r="G94" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H94" s="7" t="s">
         <v>11</v>
       </c>
       <c r="I94" s="8" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
     </row>
     <row r="95" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A95" s="17" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="B95" s="4" t="s">
+        <v>266</v>
+      </c>
+      <c r="C95" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D95" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="E95" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="F95" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G95" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H95" s="12" t="s">
         <v>267</v>
       </c>
-      <c r="C95" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="D95" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="E95" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="F95" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="G95" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="H95" s="12" t="s">
+      <c r="I95" s="10" t="s">
         <v>268</v>
       </c>
-      <c r="I95" s="10" t="s">
+      <c r="J95" s="10" t="s">
         <v>269</v>
-      </c>
-      <c r="J95" s="10" t="s">
-        <v>270</v>
       </c>
     </row>
     <row r="96" spans="1:10" s="9" customFormat="1" ht="20.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A96" s="18" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="B96" s="6" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="C96" s="4" t="s">
         <v>7</v>
@@ -4372,22 +4372,22 @@
         <v>9</v>
       </c>
       <c r="G96" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H96" s="7" t="s">
         <v>14</v>
-      </c>
-      <c r="H96" s="7" t="s">
-        <v>15</v>
       </c>
       <c r="I96" s="4"/>
       <c r="J96" s="8" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="97" spans="1:10" s="9" customFormat="1" ht="20.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A97" s="18" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="B97" s="6" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="C97" s="4" t="s">
         <v>7</v>
@@ -4402,22 +4402,22 @@
         <v>9</v>
       </c>
       <c r="G97" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H97" s="7" t="s">
         <v>14</v>
-      </c>
-      <c r="H97" s="7" t="s">
-        <v>15</v>
       </c>
       <c r="I97" s="4"/>
       <c r="J97" s="8" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="98" spans="1:10" s="9" customFormat="1" ht="20.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A98" s="18" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="B98" s="6" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="C98" s="4" t="s">
         <v>7</v>
@@ -4432,22 +4432,22 @@
         <v>9</v>
       </c>
       <c r="G98" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H98" s="7" t="s">
         <v>14</v>
-      </c>
-      <c r="H98" s="7" t="s">
-        <v>15</v>
       </c>
       <c r="I98" s="4"/>
       <c r="J98" s="8" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="99" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A99" s="11" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="B99" s="4" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C99" s="4" t="s">
         <v>7</v>
@@ -4462,24 +4462,24 @@
         <v>9</v>
       </c>
       <c r="G99" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H99" s="7">
         <v>52</v>
       </c>
       <c r="I99" s="8" t="s">
+        <v>291</v>
+      </c>
+      <c r="J99" s="8" t="s">
         <v>292</v>
-      </c>
-      <c r="J99" s="8" t="s">
-        <v>293</v>
       </c>
     </row>
     <row r="100" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A100" s="11" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="B100" s="4" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="C100" s="4" t="s">
         <v>7</v>
@@ -4494,24 +4494,24 @@
         <v>9</v>
       </c>
       <c r="G100" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H100" s="7">
         <v>45</v>
       </c>
       <c r="I100" s="8" t="s">
+        <v>291</v>
+      </c>
+      <c r="J100" s="8" t="s">
         <v>292</v>
-      </c>
-      <c r="J100" s="8" t="s">
-        <v>293</v>
       </c>
     </row>
     <row r="101" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A101" s="11" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="B101" s="4" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="C101" s="4" t="s">
         <v>7</v>
@@ -4526,24 +4526,24 @@
         <v>9</v>
       </c>
       <c r="G101" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H101" s="7">
         <v>40</v>
       </c>
       <c r="I101" s="8" t="s">
+        <v>291</v>
+      </c>
+      <c r="J101" s="8" t="s">
         <v>292</v>
-      </c>
-      <c r="J101" s="8" t="s">
-        <v>293</v>
       </c>
     </row>
     <row r="102" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A102" s="11" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="B102" s="4" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="C102" s="4" t="s">
         <v>7</v>
@@ -4558,16 +4558,16 @@
         <v>9</v>
       </c>
       <c r="G102" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H102" s="7">
         <v>15</v>
       </c>
       <c r="I102" s="8" t="s">
+        <v>291</v>
+      </c>
+      <c r="J102" s="8" t="s">
         <v>292</v>
-      </c>
-      <c r="J102" s="8" t="s">
-        <v>293</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Completed filling out the T/F values in the 3 auto log columns
</commit_message>
<xml_diff>
--- a/SWTest/Navigator.xlsx
+++ b/SWTest/Navigator.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\u245231\Quan_Vo\Local_Dev\complete-pandas-tutorial\SWTest\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7E00F4F-E67E-4FB4-A1BB-B4F89A089B70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{234B2D15-438E-49B0-8B7B-03BA599F287D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="692" uniqueCount="307">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="692" uniqueCount="308">
   <si>
     <t>Display Types</t>
   </si>
@@ -1011,6 +1011,9 @@
   </si>
   <si>
     <t>Log event if SOT (start of trip) slected</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Log event if parameter value changes. </t>
   </si>
 </sst>
 </file>
@@ -2555,7 +2558,7 @@
         <v>11</v>
       </c>
       <c r="I35" s="8" t="s">
-        <v>78</v>
+        <v>307</v>
       </c>
       <c r="J35" s="4" t="s">
         <v>108</v>

</xml_diff>